<commit_message>
Add CSV support and optional attachment feature (Closes #1)
</commit_message>
<xml_diff>
--- a/TEST.xlsx
+++ b/TEST.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76F17D3E-8F76-4AA7-B270-73490B3783FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>email</t>
   </si>
@@ -30,19 +31,16 @@
     <t>full_name</t>
   </si>
   <si>
-    <t>Rohan</t>
+    <t>PJ147_0001</t>
   </si>
   <si>
-    <t>PJ147_0018</t>
-  </si>
-  <si>
-    <t>Rohanjatasra@gmail.com</t>
+    <t>technicalboyprince@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -380,16 +378,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="34" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="34" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="34" style="2"/>
     <col min="3" max="3" width="19" style="2" customWidth="1"/>
     <col min="4" max="16384" width="34" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -400,26 +398,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="3" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>